<commit_message>
Match lot code example to data file
</commit_message>
<xml_diff>
--- a/practice/answers/s1_q16.xlsx
+++ b/practice/answers/s1_q16.xlsx
@@ -482,10 +482,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
@@ -600,18 +600,77 @@
       </c>
     </row>
     <row r="13" ht="18" customHeight="1"/>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>7,675 against 15,350. The total row already holds the five fields, so including it adds the whole farm a second time. Leave a blank row under a table, or look at what the range highlights before pressing Enter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1"/>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Two fields added later</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Xena</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>1615</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Yardley</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1"/>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>The original five-row SUM</t>
+        </is>
+      </c>
+      <c r="C18" s="10">
+        <f>SUM(B5:B9)</f>
+        <v/>
+      </c>
+      <c r="D18" s="9">
+        <f>_xlfn.FORMULATEXT(C18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>SUM over all seven</t>
+        </is>
+      </c>
+      <c r="C19" s="10">
+        <f>SUM(B5:B9,B15:B16)</f>
+        <v/>
+      </c>
+      <c r="D19" s="9">
+        <f>_xlfn.FORMULATEXT(C19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1"/>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>7,675 / 15,350 / 7,675 / 10,230. A range can reach too far and swallow the total row, doubling the answer, or fall short and miss rows added later. Neither raises an error -- both just return a plausible number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A21:D21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>